<commit_message>
August 2026 updates from CVO monitoring: housing queue, ownerless lists, grain harvest, Voin figures
- Who Gets a Home: 21 compensation decisions annulled 17 August, 100+ under
  review, six-month title extinguishment, Gosuslugi and Rosreestr gating.
- Taking Homes: 19 August ownerless package (Order No. 243, 345 flats listed
  by whole buildings with cadastral numbers), Resolution No. 1505, deadline
  extended to 1 January 2027.
- Occupation Discount: record 2026 harvest, 28.5% of declared grain by mass
  under cancelled declarations, federal transport compensation, weak exports.
- Youth militarisation dataset: Voin and Avangard entries carry 2024 to 2026
  summer-session figures.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
+++ b/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
@@ -1478,12 +1478,12 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Not stated; at least 70 students at the first camp (Henichesk)</t>
+          <t>Not stated for the occupied territories as a whole; at least 70 students at the first camp (Henichesk). Summer sessions across Russia: 10,905 cadets in 2024 and 12,935 in 78 sessions in 2025. From the occupied territories: over 300 children from Donetsk, Luhansk, Zaporizhzhia and Kherson oblasts in a single 2024 session; 781 from the "DNR" and over 140 from the "LNR" in one 2025 session; at least 91 from Zaporizhzhia oblast and 123 from Luhansk oblast confirmed in two documented 2026 groups</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/</t>
+          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/; Centre for the Study of Occupation study of the Voin summer network, Mariupol monitoring, August 2026</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1494,7 +1494,7 @@
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>Director I. V. Kazarezov from February 2024; national umbrella structure for the networks in entries 25 to 30.</t>
+          <t>Director I. V. Kazarezov from February 2024; national umbrella structure for the networks in entries 25 to 30. The Avangard defence and sports camp in Volgograd oblast is the main hub for Voin summer sessions: about 2,200 to 2,600 adolescents in 2024, 3,400 in 2025, about 4,500 planned for 2026. Programmes combine drone operation, tactical medicine, engineering, communications, weapons training and security fundamentals.</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>A plot of more than 10 hectares was taken from the former Gagarin camp for construction; UK sanctions (FCDO, 19 November 2024, together with Yunarmiya).</t>
+          <t>A plot of more than 10 hectares was taken from the former Gagarin camp for construction; UK sanctions (FCDO, 19 November 2024, together with Yunarmiya). The Avangard camp in Volgograd oblast, the network's main site for children from the occupied territories, took about 2,200 to 2,600 adolescents in 2024 and 3,400 in 2025, with about 4,500 planned for 2026; the first 2026 session had about 900 cadets and the final August 2026 session about 1,200 from 55 regions (Centre for the Study of Occupation, August 2026).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add DOC-152: CSO report on the military-ideological training of children in the occupied territories
Centre for the Study of Occupation analytical report of 17 September 2026,
published in full as a hub page with its seven graphics and 54 linked
Russian sources. Forward links from the Voin Generation briefing and the
youth militarisation dataset; seven dataset entries refreshed with the
report's figures.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
+++ b/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
@@ -614,12 +614,12 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>3 million children (Russia-wide figure); 136,000 teachers</t>
+          <t>3 million children (Russia-wide figure); 136,000 teachers; occupied Zaporizhzhia oblast: 97 schools, 626 class-teams, 10,154 pupils at the start of the 2025/26 school year; over 500 first-graders inducted in occupied Donetsk on 1 September 2026</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>https://orlyatarussia.ru/; https://investigator.org.ua/ua/investigations/266966/</t>
+          <t>https://orlyatarussia.ru/; https://investigator.org.ua/ua/investigations/266966/; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Not stated for the occupied territories as a whole; at least 70 students at the first camp (Henichesk). Summer sessions across Russia: 10,905 cadets in 2024 and 12,935 in 78 sessions in 2025. From the occupied territories: over 300 children from Donetsk, Luhansk, Zaporizhzhia and Kherson oblasts in a single 2024 session; 781 from the "DNR" and over 140 from the "LNR" in one 2025 session; at least 91 from Zaporizhzhia oblast and 123 from Luhansk oblast confirmed in two documented 2026 groups</t>
+          <t>10,381 trained participants across the four occupied oblasts by 11 March 2026 (occupied Donetsk 3,708, Luhansk 3,126, Zaporizhzhia 1,935, Kherson 1,612; ages 14 to 35, so not a child-only figure). Time of Young Heroes camps for ages 14 to 17 across the whole VOIN network: 9,158 in 2023, 10,905 in 2024, 12,935 in 78 sessions in 2025. From the occupied territories: over 300 children in a single 2024 session; 781 from the "DNR" and over 140 from the "LNR" in one 2025 session; at least 91 from Zaporizhzhia oblast and 123 from Luhansk oblast confirmed in two 2026 groups. At least 70 students at the first camp (Henichesk)</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/; Centre for the Study of Occupation study of the Voin summer network, Mariupol monitoring, August 2026</t>
+          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/; Centre for the Study of Occupation study of the Voin summer network, Mariupol monitoring, August 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -2686,12 +2686,12 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>At least 50,000 in the occupied territories (2024 to 2025): LNR 102 detachments in 24 municipalities, over 6,000 members; DNR over 5,000; Crimea 15,000 (from 1,500 in 2017); Russia-wide about 1.8 million</t>
+          <t>At least 50,000 in the occupied territories (2024 to 2025 aggregate estimate). Occupied Donetsk, post-re-registration series: over 5,000 (November 2024), over 5,500 (May 2025), 6,347 (28 January 2026), about 7,000 (May 2026), with up to 190 detachments in 18 municipalities, six Yunarmiya Houses operating and 14 more planned; the 2023 figure of 5,500 and the September 2024 figure of 4,100 are not comparable because of the 2023 re-registration. Mariupol: first detachment 9 May 2022, about 10 detachments and over 200 active participants by May 2025, Yunarmiya House opened 2024. LNR: 102 detachments in 24 municipalities, over 6,000 members cited in 2024 to 2025 (includes graduates and older age groups). Occupied Zaporizhzhia: 28 detachments, 355 participants (1 September 2025). Crimea 15,000 (from 1,500 in 2017). Russia-wide about 1.8 million</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>https://yunarmy.ru/; https://investigator.org.ua/ua/investigations/266966/; Barbieri, Ethnopolitics 23(5), 2024, pp. 515 to 536; Hird et al., ISW, 2024</t>
+          <t>https://yunarmy.ru/; https://investigator.org.ua/ua/investigations/266966/; Barbieri, Ethnopolitics 23(5), 2024, pp. 515 to 536; Hird et al., ISW, 2024; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Mariupol 1,500 children; Zaporizhzhia oblast 19,000 children; LNR over 70,000 events per school year</t>
+          <t>Occupied Zaporizhzhia: over 14,000 participants (end 2024), over 23,000 activists (end 2025), 189 primary branches (start of 2025/26); occupied Donetsk: 27,000 participants (July 2026) with a stated goal of every second schoolchild; Mariupol 1,500 children (40 branches in 27 institutions); LNR about 3,500 detachments and over 70,000 events per school year; occupied Kherson: over 1,500 events and 47 projects in 2025</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/news/uk-sanctions-actors-forcibly-deporting-indoctrinating-and-militarising-ukrainian-children; Hird et al., ISW, 2024; McGlynn et al., Capturing the Minds, 2026</t>
+          <t>https://www.gov.uk/government/news/uk-sanctions-actors-forcibly-deporting-indoctrinating-and-militarising-ukrainian-children; Hird et al., ISW, 2024; McGlynn et al., Capturing the Minds, 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -5830,12 +5830,12 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Crimea: 244 classes in 78 schools (2023/24)</t>
+          <t>Crimea: 244 classes in 78 schools (2023/24); occupied Zaporizhzhia, September 2025: 11 cadet classes with 279 pupils and four profile classes linked to the Investigative Committee, Emergencies Ministry and Interior Ministry with 108 pupils, 387 in total</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>Crimean Human Rights House / Crimean Human Rights Group / Regional Centre for Human Rights / Almenda / ZMINA, 2021, pp. 63 to 65; Crimean Human Rights Group, 12 June 2020, https://crimeahrg.org/uk/rosijske-kadetstvo-zamist-krimskogo-ditinstva/; Save Ukraine / War Child UK, 2025</t>
+          <t>Crimean Human Rights House / Crimean Human Rights Group / Regional Centre for Human Rights / Almenda / ZMINA, 2021, pp. 63 to 65; Crimean Human Rights Group, 12 June 2020, https://crimeahrg.org/uk/rosijske-kadetstvo-zamist-krimskogo-ditinstva/; Save Ukraine / War Child UK, 2025; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -6006,12 +6006,12 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Not stated (covers all pupils in the relevant years)</t>
+          <t>Not stated (covers all pupils in the relevant years); OBZR classrooms equipped in 513 schools in occupied Donetsk during 2025</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>Russian Ministry of Education programme document on basic military training for years 10 to 11; TOT Insights, Education and Militarisation analytical brief, section 2.4; TOT Insights, The Voin Generation (2026), section II</t>
+          <t>Russian Ministry of Education programme document on basic military training for years 10 to 11; TOT Insights, Education and Militarisation analytical brief, section 2.4; TOT Insights, The Voin Generation (2026), section II; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
@@ -6092,12 +6092,12 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Mariupol: over 2,600 children (first half of 2025); Zaporizhzhia oblast: over 2,000 planned</t>
+          <t>Occupied Zaporizhzhia: about 860 in 2024, over 2,000 in 2025, at least 2,000 targeted for 2026; occupied Kherson: over 600 in 2024, over 1,200 from 60 educational institutions in 2025; Mariupol: over 2,600 children (first half of 2025)</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Centre for the Study of Occupation monitoring, Mariupol and Luhansk oblast, 2025, and Mariupol, June 2026</t>
+          <t>Centre for the Study of Occupation monitoring, Mariupol and Luhansk oblast, 2025, and Mariupol, June 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Withdraw DOC-152 (CSO report on military-ideological training of children)
Content to be used in another publication. Page removed, catalogue entry
deleted, forward links from the Voin Generation briefing, the youth
militarisation dataset page and the Education theme card removed, and the
dataset restored to its 16 September state so no entry cites the withdrawn
page.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
+++ b/data/youth-militarisation/tot_youth_militarisation_dataset_en.xlsx
@@ -614,12 +614,12 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>3 million children (Russia-wide figure); 136,000 teachers; occupied Zaporizhzhia oblast: 97 schools, 626 class-teams, 10,154 pupils at the start of the 2025/26 school year; over 500 first-graders inducted in occupied Donetsk on 1 September 2026</t>
+          <t>3 million children (Russia-wide figure); 136,000 teachers</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>https://orlyatarussia.ru/; https://investigator.org.ua/ua/investigations/266966/; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>https://orlyatarussia.ru/; https://investigator.org.ua/ua/investigations/266966/</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>10,381 trained participants across the four occupied oblasts by 11 March 2026 (occupied Donetsk 3,708, Luhansk 3,126, Zaporizhzhia 1,935, Kherson 1,612; ages 14 to 35, so not a child-only figure). Time of Young Heroes camps for ages 14 to 17 across the whole VOIN network: 9,158 in 2023, 10,905 in 2024, 12,935 in 78 sessions in 2025. From the occupied territories: over 300 children in a single 2024 session; 781 from the "DNR" and over 140 from the "LNR" in one 2025 session; at least 91 from Zaporizhzhia oblast and 123 from Luhansk oblast confirmed in two 2026 groups. At least 70 students at the first camp (Henichesk)</t>
+          <t>Not stated for the occupied territories as a whole; at least 70 students at the first camp (Henichesk). Summer sessions across Russia: 10,905 cadets in 2024 and 12,935 in 78 sessions in 2025. From the occupied territories: over 300 children from Donetsk, Luhansk, Zaporizhzhia and Kherson oblasts in a single 2024 session; 781 from the "DNR" and over 140 from the "LNR" in one 2025 session; at least 91 from Zaporizhzhia oblast and 123 from Luhansk oblast confirmed in two documented 2026 groups</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/; Centre for the Study of Occupation study of the Voin summer network, Mariupol monitoring, August 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>https://crvsp.ru/center; https://lb.ua/blog/koalitsiia_ua5am/620037_voini_rosiyskogo_rezhimu_yak.html; https://war-sanctions.gur.gov.ua/kidnappers/companies/13074; https://1news.zp.ua/; Centre for the Study of Occupation study of the Voin summer network, Mariupol monitoring, August 2026</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -2686,12 +2686,12 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>At least 50,000 in the occupied territories (2024 to 2025 aggregate estimate). Occupied Donetsk, post-re-registration series: over 5,000 (November 2024), over 5,500 (May 2025), 6,347 (28 January 2026), about 7,000 (May 2026), with up to 190 detachments in 18 municipalities, six Yunarmiya Houses operating and 14 more planned; the 2023 figure of 5,500 and the September 2024 figure of 4,100 are not comparable because of the 2023 re-registration. Mariupol: first detachment 9 May 2022, about 10 detachments and over 200 active participants by May 2025, Yunarmiya House opened 2024. LNR: 102 detachments in 24 municipalities, over 6,000 members cited in 2024 to 2025 (includes graduates and older age groups). Occupied Zaporizhzhia: 28 detachments, 355 participants (1 September 2025). Crimea 15,000 (from 1,500 in 2017). Russia-wide about 1.8 million</t>
+          <t>At least 50,000 in the occupied territories (2024 to 2025): LNR 102 detachments in 24 municipalities, over 6,000 members; DNR over 5,000; Crimea 15,000 (from 1,500 in 2017); Russia-wide about 1.8 million</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>https://yunarmy.ru/; https://investigator.org.ua/ua/investigations/266966/; Barbieri, Ethnopolitics 23(5), 2024, pp. 515 to 536; Hird et al., ISW, 2024; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>https://yunarmy.ru/; https://investigator.org.ua/ua/investigations/266966/; Barbieri, Ethnopolitics 23(5), 2024, pp. 515 to 536; Hird et al., ISW, 2024</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Occupied Zaporizhzhia: over 14,000 participants (end 2024), over 23,000 activists (end 2025), 189 primary branches (start of 2025/26); occupied Donetsk: 27,000 participants (July 2026) with a stated goal of every second schoolchild; Mariupol 1,500 children (40 branches in 27 institutions); LNR about 3,500 detachments and over 70,000 events per school year; occupied Kherson: over 1,500 events and 47 projects in 2025</t>
+          <t>Mariupol 1,500 children; Zaporizhzhia oblast 19,000 children; LNR over 70,000 events per school year</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/news/uk-sanctions-actors-forcibly-deporting-indoctrinating-and-militarising-ukrainian-children; Hird et al., ISW, 2024; McGlynn et al., Capturing the Minds, 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>https://www.gov.uk/government/news/uk-sanctions-actors-forcibly-deporting-indoctrinating-and-militarising-ukrainian-children; Hird et al., ISW, 2024; McGlynn et al., Capturing the Minds, 2026</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -5830,12 +5830,12 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Crimea: 244 classes in 78 schools (2023/24); occupied Zaporizhzhia, September 2025: 11 cadet classes with 279 pupils and four profile classes linked to the Investigative Committee, Emergencies Ministry and Interior Ministry with 108 pupils, 387 in total</t>
+          <t>Crimea: 244 classes in 78 schools (2023/24)</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>Crimean Human Rights House / Crimean Human Rights Group / Regional Centre for Human Rights / Almenda / ZMINA, 2021, pp. 63 to 65; Crimean Human Rights Group, 12 June 2020, https://crimeahrg.org/uk/rosijske-kadetstvo-zamist-krimskogo-ditinstva/; Save Ukraine / War Child UK, 2025; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>Crimean Human Rights House / Crimean Human Rights Group / Regional Centre for Human Rights / Almenda / ZMINA, 2021, pp. 63 to 65; Crimean Human Rights Group, 12 June 2020, https://crimeahrg.org/uk/rosijske-kadetstvo-zamist-krimskogo-ditinstva/; Save Ukraine / War Child UK, 2025</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -6006,12 +6006,12 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Not stated (covers all pupils in the relevant years); OBZR classrooms equipped in 513 schools in occupied Donetsk during 2025</t>
+          <t>Not stated (covers all pupils in the relevant years)</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>Russian Ministry of Education programme document on basic military training for years 10 to 11; TOT Insights, Education and Militarisation analytical brief, section 2.4; TOT Insights, The Voin Generation (2026), section II; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>Russian Ministry of Education programme document on basic military training for years 10 to 11; TOT Insights, Education and Militarisation analytical brief, section 2.4; TOT Insights, The Voin Generation (2026), section II</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
@@ -6092,12 +6092,12 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Occupied Zaporizhzhia: about 860 in 2024, over 2,000 in 2025, at least 2,000 targeted for 2026; occupied Kherson: over 600 in 2024, over 1,200 from 60 educational institutions in 2025; Mariupol: over 2,600 children (first half of 2025)</t>
+          <t>Mariupol: over 2,600 children (first half of 2025); Zaporizhzhia oblast: over 2,000 planned</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Centre for the Study of Occupation monitoring, Mariupol and Luhansk oblast, 2025, and Mariupol, June 2026; Centre for the Study of Occupation, The System of Military-Ideological Training of Children in the Temporarily Occupied Territories of Ukraine, 17 September 2026 (https://totinsights.org/briefings/cvo_militarisation_children.html)</t>
+          <t>Centre for the Study of Occupation monitoring, Mariupol and Luhansk oblast, 2025, and Mariupol, June 2026</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">

</xml_diff>